<commit_message>
Credit IDP survey pollster as OPERSO - Operatyvna Sotsiolohiia with link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/idp-survey/idp_survey_2026.xlsx
+++ b/data/idp-survey/idp_survey_2026.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Operativna Sotsiolohiya (Оперативна соціологія)</t>
+          <t>OPERSO - Operatyvna Sotsiolohiia (Оперативна соціологія), https://operso.com.ua/</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>TOT Insights and Operativna Sotsiolohiya. IDP Attitudes Survey 2026. October 2026. https://totinsights.org/idp-survey-2026.html</t>
+          <t>TOT Insights and OPERSO - Operatyvna Sotsiolohiia. IDP Attitudes Survey 2026. October 2026. https://totinsights.org/idp-survey-2026.html</t>
         </is>
       </c>
     </row>

</xml_diff>